<commit_message>
Removed generic link text
</commit_message>
<xml_diff>
--- a/docassemble/MAEvictionDefense/data/sources/eviction_es.xlsx
+++ b/docassemble/MAEvictionDefense/data/sources/eviction_es.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1219"/>
+  <dimension ref="A1:H1223"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25.7109375" customWidth="1" min="1" max="1"/>
@@ -18258,7 +18258,7 @@
       </c>
       <c r="D421" s="2" t="inlineStr">
         <is>
-          <t>06affba7ad2203d850a91c6af6819f61</t>
+          <t>575ad08957cfe9bd85d7f94d8711ed35</t>
         </is>
       </c>
       <c r="E421" s="2" t="inlineStr">
@@ -18276,7 +18276,7 @@
           <t xml:space="preserve">You can continue this interview on another device, or share it with 
 someone who will help you finish it. Choose any of the options below to share
 the interview.
-Right-click and copy [this link](${interview_url()}).
+Right-click and copy [the link to your interview](${interview_url()}).
 % if device() and not device().is_mobile:
 Use your phone's camera to point at this barcode. Click the link that appears
 in the camera's viewfinder.
@@ -18291,7 +18291,7 @@
         <is>
           <t xml:space="preserve">Puedes continuar esta entrevista en otro dispositivo o compartirla con alguien que te ayude a terminarla.  Escoge cualquiera de las siguientes opciones para compartir
 la entrevista.
-Haz clic derecho y copia [este enlace](${interview_url()}).
+Haz clic derecho y copia [el enlace a tu entrevista](${interview_url()}).
 % if device() and not device().is_mobile:
 Use la cámara de tu teléfono para escanar este código de barras. 
  Haz clic en el enlace que aparece en el visor de la cámara.
@@ -40554,7 +40554,7 @@
       </c>
       <c r="D949" s="2" t="inlineStr">
         <is>
-          <t>405a7c1de4db0b51f49baacb5de85580</t>
+          <t>8d80904edef43f2eedc35a288289b349</t>
         </is>
       </c>
       <c r="E949" s="2" t="inlineStr">
@@ -40584,7 +40584,7 @@
   ${landlord.name}.
 % endif
 You also need to send a copy of the motion to ${court}.
-Learn more and continue the form online [here](${interview_url()}) or download
+Learn more and [continue the form online](${interview_url()}) or download
 the PDF here: https://gbls.org/tactics/compel.
 </t>
         </is>
@@ -40603,7 +40603,7 @@
   ${landlord.name}.
 % endif
 También debes hacer llegar una copia a los tribunales ${court}.
-Aprende más y continúa con el formulario en línea [aquí](${interview_url()}) o descarga el PDF aquí https://gbls.org/tactics/compel.
+Aprende más y [continúa con el formulario en línea](${interview_url()}) o descarga el PDF aquí https://gbls.org/tactics/compel.
 </t>
         </is>
       </c>
@@ -40881,7 +40881,7 @@
       </c>
       <c r="D955" s="2" t="inlineStr">
         <is>
-          <t>26fd8aed4ec30f78c45f916032146cd5</t>
+          <t>cec6553a0281b8bd2f9e4a1f35f60906</t>
         </is>
       </c>
       <c r="E955" s="2" t="inlineStr">
@@ -40898,14 +40898,14 @@
         <is>
           <t xml:space="preserve">Someone who was completing an interview using Massachusetts Defense for
 Eviction (MADE) sent you this link.
-Click [here](${interview_url()}) to keep working on the interview.
+[Keep working on the interview](${interview_url()}).
 </t>
         </is>
       </c>
       <c r="H955" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Alguien que estaba completando una entrevista usando la Defensa de Desalojo de Massachusetts (MADE) le envió este enlace.
-[Haga clic aquí](${interview_url()}) para seguir trabajando en la entrevista.
+          <t xml:space="preserve">Alguien que estaba completando una entrevista usando la Defensa de Desalojo de Massachusetts (MADE) te envió este enlace.
+[Sigue trabajando en la entrevista](${interview_url()}).
 </t>
         </is>
       </c>
@@ -53226,6 +53226,208 @@
         </is>
       </c>
     </row>
+    <row r="1220">
+      <c r="A1220" t="inlineStr">
+        <is>
+          <t>docassemble.MAEvictionDefense:data/questions/eviction.en.yml</t>
+        </is>
+      </c>
+      <c r="B1220" t="inlineStr">
+        <is>
+          <t>method of service</t>
+        </is>
+      </c>
+      <c r="C1220" t="n">
+        <v>12</v>
+      </c>
+      <c r="D1220" t="inlineStr">
+        <is>
+          <t>a2beb488f5408ec32ba0f33f24c6c5e1</t>
+        </is>
+      </c>
+      <c r="E1220" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="F1220" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="G1220" t="inlineStr">
+        <is>
+          <t>By hand</t>
+        </is>
+      </c>
+      <c r="H1220" t="inlineStr">
+        <is>
+          <t>En mano</t>
+        </is>
+      </c>
+    </row>
+    <row r="1221">
+      <c r="A1221" t="inlineStr">
+        <is>
+          <t>docassemble.MAEvictionDefense:data/questions/eviction.en.yml</t>
+        </is>
+      </c>
+      <c r="B1221" t="inlineStr">
+        <is>
+          <t>method of service</t>
+        </is>
+      </c>
+      <c r="C1221" t="n">
+        <v>13</v>
+      </c>
+      <c r="D1221" t="inlineStr">
+        <is>
+          <t>dfc27ef27b631b0e7114573a439c3180</t>
+        </is>
+      </c>
+      <c r="E1221" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="F1221" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="G1221" t="inlineStr">
+        <is>
+          <t>By email</t>
+        </is>
+      </c>
+      <c r="H1221" t="inlineStr">
+        <is>
+          <t>Por correo electrónico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1222">
+      <c r="A1222" t="inlineStr">
+        <is>
+          <t>docassemble.MAEvictionDefense:data/questions/eviction.en.yml</t>
+        </is>
+      </c>
+      <c r="B1222" t="inlineStr">
+        <is>
+          <t>method of service</t>
+        </is>
+      </c>
+      <c r="C1222" t="n">
+        <v>14</v>
+      </c>
+      <c r="D1222" t="inlineStr">
+        <is>
+          <t>409b1ef3ad4fe98ad063fb3026c6b250</t>
+        </is>
+      </c>
+      <c r="E1222" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="F1222" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="G1222" t="inlineStr">
+        <is>
+          <t>By mail</t>
+        </is>
+      </c>
+      <c r="H1222" t="inlineStr">
+        <is>
+          <t>Por correo postal</t>
+        </is>
+      </c>
+    </row>
+    <row r="1223">
+      <c r="A1223" t="inlineStr">
+        <is>
+          <t>docassemble.MAEvictionDefense:data/questions/eviction.en.yml</t>
+        </is>
+      </c>
+      <c r="B1223" t="inlineStr">
+        <is>
+          <t>method of service</t>
+        </is>
+      </c>
+      <c r="C1223" t="n">
+        <v>15</v>
+      </c>
+      <c r="D1223" t="inlineStr">
+        <is>
+          <t>966afd80841437ca4adfcf8f54bfab2a</t>
+        </is>
+      </c>
+      <c r="E1223" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="F1223" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="G1223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">You must give a copy of the forms we are working on to your landlord or their 
+attorney. 
+% if case.hearing_date_assigned:
+They need to _get_ the forms no later than 
+**${format_date(case.answer_date)}**.
+% if answer_date_is_holiday:
+Because ${case.answer_date} is ${answer_date_holiday}, you can
+deliver it the next weekday after ${answer_date_holiday}.
+% endif
+% else:
+Give a copy to your landlord or their attorney as soon as you can.
+% endif
+Deliver it in person
+if you can. If your landlord has a lawyer, you can email it to the lawyer.
+If your landlord does not have a lawyer, ask them first before you email it. 
+% if format_date(case.answer_date) == format_date(today()):
+It's too late to mail the paperwork.
+% else:
+Only mail it if you know
+your landlord will get it on or before ${format_date(case.answer_date)}.
+% endif
+</t>
+        </is>
+      </c>
+      <c r="H1223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tienes que darle una copia de los formularios en los que estamos trabajando a tu dueño o a su 
+abogado. 
+% if case.hearing_date_assigned:
+Tienen que _recibir_ los formularios a más tardar el 
+**${format_date(case.answer_date)}**.
+% if answer_date_is_holiday:
+Como el ${case.answer_date} es ${answer_date_holiday}, puedes
+entregarlo el siguiente día hábil después del ${answer_date_holiday}.
+% endif
+% else:
+Dale una copia a tu dueño o a su abogado lo antes posible.
+% endif
+Entrégalo en persona
+si puedes. Si tu dueño tiene abogado, se lo puedes mandar por correo electrónico al abogado.
+Si tu dueño no tiene abogado, pídele permiso antes de mandárselo por correo electrónico. 
+% if format_date(case.answer_date) == format_date(today()):
+Ya es demasiado tarde para mandar los documentos por correo postal.
+% else:
+Mándalo por correo solo si sabes que
+tu dueño lo va a recibir el ${format_date(case.answer_date)} o antes.
+% endif
+</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>